<commit_message>
fix(m4): member 213 owed nothing — deuda.xlsx corrected, control totals 118/3076
The workbook listed 4 fees for 2024 on member 213 by mistake. Mariano fixed
the file on 22/08/2026; the import's control totals (EXPECTED_DEBTORS,
EXPECTED_TOTAL_FEES) and every document that quotes them follow: 119 -> 118
debtors, 3080 -> 3076 fees, 8 -> 7 vigentes with debt.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/deuda.xlsx
+++ b/datos/deuda.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\ciudadela\datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BA92B4F-A176-49BE-A66E-2E49DC187335}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A420CF1-3059-4C3F-A639-F89F6F28F23A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{33464C6B-A528-44FF-AC66-54FA3E9E2F8E}"/>
   </bookViews>
@@ -7411,7 +7411,7 @@
         <v>0</v>
       </c>
       <c r="G198" s="36">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H198" s="38">
         <v>0</v>

</xml_diff>